<commit_message>
Update Dental CBCT templates for improved data representation and consistency
- Revised the structure of the Dental CBCT test data templates, including changes to header labels and measurement parameters for radiation leakage tests, enhancing clarity and consistency.
- Standardized the format of tolerance operators and measurement units across templates, improving overall reporting quality.
- Updated the export functions for generating Excel files to ensure accurate data handling and organization.
</commit_message>
<xml_diff>
--- a/public/templates/Dental_CBCT_Template.xlsx
+++ b/public/templates/Dental_CBCT_Template.xlsx
@@ -398,26 +398,45 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J39"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="18.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:L38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>TEST: ACCURACY OF OPERATING POTENTIAL</v>
       </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+      <c r="G1" t="str">
+        <v/>
+      </c>
+      <c r="H1" t="str">
+        <v/>
+      </c>
+      <c r="I1" t="str">
+        <v/>
+      </c>
+      <c r="J1" t="str">
+        <v/>
+      </c>
+      <c r="K1" t="str">
+        <v/>
+      </c>
+      <c r="L1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -435,6 +454,27 @@
       <c r="E2" t="str">
         <v>Remarks</v>
       </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -452,6 +492,27 @@
       <c r="E3" t="str">
         <v/>
       </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -469,6 +530,27 @@
       <c r="E4" t="str">
         <v/>
       </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -486,11 +568,103 @@
       <c r="E5" t="str">
         <v/>
       </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v/>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
         <v>TEST: TOTAL FILTRATION</v>
       </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -505,6 +679,30 @@
       <c r="D8" t="str">
         <v>At kVp</v>
       </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -519,11 +717,106 @@
       <c r="D9" t="str">
         <v>80</v>
       </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
         <v>TEST: ACCURACY OF IRRADIATION TIME</v>
       </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -544,6 +837,24 @@
       <c r="F12" t="str">
         <v>10</v>
       </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -555,6 +866,33 @@
       <c r="C13" t="str">
         <v>% Error</v>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -566,6 +904,33 @@
       <c r="C14" t="str">
         <v/>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -577,11 +942,109 @@
       <c r="C15" t="str">
         <v/>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v/>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
         <v>TEST: LINEARITY OF mA LOADING</v>
       </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -602,6 +1065,24 @@
       <c r="F18" t="str">
         <v>0.1</v>
       </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -622,6 +1103,24 @@
       <c r="F19" t="str">
         <v>mR/mAs</v>
       </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -642,6 +1141,24 @@
       <c r="F20" t="str">
         <v/>
       </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -662,11 +1179,100 @@
       <c r="F21" t="str">
         <v/>
       </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v/>
+      </c>
+      <c r="B22" t="str">
+        <v/>
+      </c>
+      <c r="C22" t="str">
+        <v/>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
         <v>TEST: CONSISTENCY OF RADIATION OUTPUT</v>
       </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v/>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -675,6 +1281,36 @@
       <c r="B24" t="str">
         <v>100</v>
       </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -701,6 +1337,18 @@
       <c r="H25" t="str">
         <v>Remarks</v>
       </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -727,36 +1375,119 @@
       <c r="H26" t="str">
         <v/>
       </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v/>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
         <v>TEST: RADIATION LEAKAGE LEVEL FROM X-RAY TUBE HOUSE</v>
       </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>FFD</v>
+        <v>kV</v>
       </c>
       <c r="B29" t="str">
+        <v>120</v>
+      </c>
+      <c r="C29" t="str">
+        <v>mA</v>
+      </c>
+      <c r="D29" t="str">
+        <v>10</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Time</v>
+      </c>
+      <c r="F29" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Workload</v>
+      </c>
+      <c r="H29" t="str">
         <v>100</v>
-      </c>
-      <c r="C29" t="str">
-        <v>kVp</v>
-      </c>
-      <c r="D29" t="str">
-        <v>120</v>
-      </c>
-      <c r="E29" t="str">
-        <v>mA</v>
-      </c>
-      <c r="F29" t="str">
-        <v>10</v>
-      </c>
-      <c r="G29" t="str">
-        <v>Time</v>
-      </c>
-      <c r="H29" t="str">
-        <v>1.0</v>
       </c>
       <c r="I29" t="str">
         <v>Tolerance</v>
@@ -764,162 +1495,249 @@
       <c r="J29" t="str">
         <v>1.0</v>
       </c>
+      <c r="K29" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="L29" t="str">
+        <v>&lt;</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Workload</v>
+        <v>Location</v>
       </c>
       <c r="B30" t="str">
-        <v>100</v>
+        <v>Front</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Back</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Left</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Right</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Max Leakage</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Remark</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Location</v>
+        <v>Tube</v>
       </c>
       <c r="B31" t="str">
-        <v>Left</v>
+        <v>0.01</v>
       </c>
       <c r="C31" t="str">
-        <v>Right</v>
+        <v>0.015</v>
       </c>
       <c r="D31" t="str">
-        <v>Top</v>
+        <v>0.012</v>
       </c>
       <c r="E31" t="str">
-        <v>Up</v>
+        <v>0.011</v>
       </c>
       <c r="F31" t="str">
-        <v>Down</v>
+        <v/>
       </c>
       <c r="G31" t="str">
-        <v>Max Leakage</v>
+        <v>mGy/h</v>
       </c>
       <c r="H31" t="str">
-        <v>Unit</v>
-      </c>
-      <c r="I31" t="str">
-        <v>Remark</v>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Front</v>
+        <v>Collimator</v>
       </c>
       <c r="B32" t="str">
-        <v>0.01</v>
+        <v>0.012</v>
       </c>
       <c r="C32" t="str">
-        <v>0.02</v>
+        <v>0.011</v>
       </c>
       <c r="D32" t="str">
-        <v>0.015</v>
+        <v>0.014</v>
       </c>
       <c r="E32" t="str">
-        <v>0.012</v>
+        <v>0.013</v>
       </c>
       <c r="F32" t="str">
-        <v>0.011</v>
+        <v/>
       </c>
       <c r="G32" t="str">
-        <v/>
+        <v>mGy/h</v>
       </c>
       <c r="H32" t="str">
         <v/>
       </c>
-      <c r="I32" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>Back</v>
-      </c>
-      <c r="B33" t="str">
-        <v>0.012</v>
-      </c>
-      <c r="C33" t="str">
-        <v>0.014</v>
-      </c>
-      <c r="D33" t="str">
-        <v>0.011</v>
-      </c>
-      <c r="E33" t="str">
-        <v>0.013</v>
-      </c>
-      <c r="F33" t="str">
-        <v>0.015</v>
-      </c>
-      <c r="G33" t="str">
-        <v/>
-      </c>
-      <c r="H33" t="str">
-        <v/>
-      </c>
-      <c r="I33" t="str">
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TEST: RADIATION PROTECTION SURVEY REPORT</v>
+      </c>
+      <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34" t="str">
+        <v/>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
+        <v/>
+      </c>
+      <c r="L34" t="str">
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>TEST: RADIATION PROTECTION SURVEY REPORT</v>
+        <v>Survey Date</v>
+      </c>
+      <c r="B35" t="str">
+        <v>2024-01-01</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Applied Current (mA)</v>
+      </c>
+      <c r="D35" t="str">
+        <v>10</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Applied Voltage (kV)</v>
+      </c>
+      <c r="F35" t="str">
+        <v>80</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Exposure Time (s)</v>
+      </c>
+      <c r="H35" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Workload (mA.min/week)</v>
+      </c>
+      <c r="J35" t="str">
+        <v>100</v>
+      </c>
+      <c r="K35" t="str">
+        <v/>
+      </c>
+      <c r="L35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Survey Date</v>
+        <v>LOCATION</v>
       </c>
       <c r="B36" t="str">
-        <v>2024-01-01</v>
+        <v>MAX. RADIATION LEVEL (MR/HR)</v>
       </c>
       <c r="C36" t="str">
-        <v>Applied Current (mA)</v>
+        <v>MR/WEEK</v>
       </c>
       <c r="D36" t="str">
-        <v>10</v>
+        <v>STATUS</v>
       </c>
       <c r="E36" t="str">
-        <v>Applied Voltage (kV)</v>
+        <v>RESULT</v>
       </c>
       <c r="F36" t="str">
-        <v>80</v>
+        <v/>
       </c>
       <c r="G36" t="str">
-        <v>Exposure Time (s)</v>
+        <v/>
       </c>
       <c r="H36" t="str">
-        <v>1.0</v>
+        <v/>
       </c>
       <c r="I36" t="str">
-        <v>Workload (mA.min/week)</v>
+        <v/>
       </c>
       <c r="J36" t="str">
-        <v>100</v>
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v/>
+      </c>
+      <c r="L36" t="str">
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>LOCATION</v>
+        <v>Control Console</v>
       </c>
       <c r="B37" t="str">
-        <v>MAX. RADIATION LEVEL (MR/HR)</v>
+        <v>0.05</v>
       </c>
       <c r="C37" t="str">
-        <v>MR/WEEK</v>
+        <v/>
       </c>
       <c r="D37" t="str">
-        <v>STATUS</v>
+        <v/>
       </c>
       <c r="E37" t="str">
-        <v>RESULT</v>
+        <v>Worker</v>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37" t="str">
+        <v/>
+      </c>
+      <c r="L37" t="str">
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Control Console</v>
+        <v>Waiting Area</v>
       </c>
       <c r="B38" t="str">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="C38" t="str">
         <v/>
@@ -928,55 +1746,72 @@
         <v/>
       </c>
       <c r="E38" t="str">
-        <v>Worker</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>Waiting Area</v>
-      </c>
-      <c r="B39" t="str">
-        <v>0.02</v>
-      </c>
-      <c r="C39" t="str">
-        <v/>
-      </c>
-      <c r="D39" t="str">
-        <v/>
-      </c>
-      <c r="E39" t="str">
         <v>Public</v>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v/>
+      </c>
+      <c r="L38" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L38"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J32"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="18.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:L31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>TEST: ACCURACY OF OPERATING POTENTIAL</v>
       </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+      <c r="G1" t="str">
+        <v/>
+      </c>
+      <c r="H1" t="str">
+        <v/>
+      </c>
+      <c r="I1" t="str">
+        <v/>
+      </c>
+      <c r="J1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -994,6 +1829,21 @@
       <c r="E2" t="str">
         <v>Remarks</v>
       </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1011,6 +1861,21 @@
       <c r="E3" t="str">
         <v/>
       </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -1028,6 +1893,21 @@
       <c r="E4" t="str">
         <v/>
       </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -1045,11 +1925,85 @@
       <c r="E5" t="str">
         <v/>
       </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v/>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
         <v>TEST: TOTAL FILTRATION</v>
       </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -1064,6 +2018,24 @@
       <c r="D8" t="str">
         <v>At kVp</v>
       </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -1078,11 +2050,88 @@
       <c r="D9" t="str">
         <v>80</v>
       </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
         <v>TEST: LINEARITY OF mAs LOADING</v>
       </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -1103,6 +2152,18 @@
       <c r="F12" t="str">
         <v>mR/mAs</v>
       </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1123,6 +2184,18 @@
       <c r="F13" t="str">
         <v/>
       </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1143,11 +2216,82 @@
       <c r="F14" t="str">
         <v/>
       </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v/>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
         <v>TEST: CONSISTENCY OF RADIATION OUTPUT</v>
       </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1156,6 +2300,30 @@
       <c r="B17" t="str">
         <v>100</v>
       </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1182,6 +2350,12 @@
       <c r="H18" t="str">
         <v>Remarks</v>
       </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1208,36 +2382,101 @@
       <c r="H19" t="str">
         <v/>
       </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
         <v>TEST: RADIATION LEAKAGE LEVEL FROM X-RAY TUBE HOUSE</v>
       </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>FFD</v>
+        <v>kV</v>
       </c>
       <c r="B22" t="str">
+        <v>120</v>
+      </c>
+      <c r="C22" t="str">
+        <v>mA</v>
+      </c>
+      <c r="D22" t="str">
+        <v>10</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Time</v>
+      </c>
+      <c r="F22" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Workload</v>
+      </c>
+      <c r="H22" t="str">
         <v>100</v>
-      </c>
-      <c r="C22" t="str">
-        <v>kVp</v>
-      </c>
-      <c r="D22" t="str">
-        <v>120</v>
-      </c>
-      <c r="E22" t="str">
-        <v>mA</v>
-      </c>
-      <c r="F22" t="str">
-        <v>10</v>
-      </c>
-      <c r="G22" t="str">
-        <v>Time</v>
-      </c>
-      <c r="H22" t="str">
-        <v>1.0</v>
       </c>
       <c r="I22" t="str">
         <v>Tolerance</v>
@@ -1245,162 +2484,225 @@
       <c r="J22" t="str">
         <v>1.0</v>
       </c>
+      <c r="K22" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="L22" t="str">
+        <v>&lt;</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Workload</v>
+        <v>Location</v>
       </c>
       <c r="B23" t="str">
-        <v>100</v>
+        <v>Front</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Back</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Left</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Right</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Max Leakage</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Remark</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Location</v>
+        <v>Tube</v>
       </c>
       <c r="B24" t="str">
-        <v>Left</v>
+        <v>0.01</v>
       </c>
       <c r="C24" t="str">
-        <v>Right</v>
+        <v>0.015</v>
       </c>
       <c r="D24" t="str">
-        <v>Top</v>
+        <v>0.012</v>
       </c>
       <c r="E24" t="str">
-        <v>Up</v>
+        <v>0.011</v>
       </c>
       <c r="F24" t="str">
-        <v>Down</v>
+        <v/>
       </c>
       <c r="G24" t="str">
-        <v>Max Leakage</v>
+        <v>mGy/h</v>
       </c>
       <c r="H24" t="str">
-        <v>Unit</v>
-      </c>
-      <c r="I24" t="str">
-        <v>Remark</v>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Front</v>
+        <v>Collimator</v>
       </c>
       <c r="B25" t="str">
-        <v>0.01</v>
+        <v>0.012</v>
       </c>
       <c r="C25" t="str">
-        <v>0.02</v>
+        <v>0.011</v>
       </c>
       <c r="D25" t="str">
-        <v>0.015</v>
+        <v>0.014</v>
       </c>
       <c r="E25" t="str">
-        <v>0.012</v>
+        <v>0.013</v>
       </c>
       <c r="F25" t="str">
-        <v>0.011</v>
+        <v/>
       </c>
       <c r="G25" t="str">
-        <v/>
+        <v>mGy/h</v>
       </c>
       <c r="H25" t="str">
         <v/>
       </c>
-      <c r="I25" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>Back</v>
-      </c>
-      <c r="B26" t="str">
-        <v>0.012</v>
-      </c>
-      <c r="C26" t="str">
-        <v>0.014</v>
-      </c>
-      <c r="D26" t="str">
-        <v>0.011</v>
-      </c>
-      <c r="E26" t="str">
-        <v>0.013</v>
-      </c>
-      <c r="F26" t="str">
-        <v>0.015</v>
-      </c>
-      <c r="G26" t="str">
-        <v/>
-      </c>
-      <c r="H26" t="str">
-        <v/>
-      </c>
-      <c r="I26" t="str">
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TEST: RADIATION PROTECTION SURVEY REPORT</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>TEST: RADIATION PROTECTION SURVEY REPORT</v>
+        <v>Survey Date</v>
+      </c>
+      <c r="B28" t="str">
+        <v>2024-01-01</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Applied Current (mA)</v>
+      </c>
+      <c r="D28" t="str">
+        <v>10</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Applied Voltage (kV)</v>
+      </c>
+      <c r="F28" t="str">
+        <v>80</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Exposure Time (s)</v>
+      </c>
+      <c r="H28" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Workload (mA.min/week)</v>
+      </c>
+      <c r="J28" t="str">
+        <v>100</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Survey Date</v>
+        <v>LOCATION</v>
       </c>
       <c r="B29" t="str">
-        <v>2024-01-01</v>
+        <v>MAX. RADIATION LEVEL (MR/HR)</v>
       </c>
       <c r="C29" t="str">
-        <v>Applied Current (mA)</v>
+        <v>MR/WEEK</v>
       </c>
       <c r="D29" t="str">
-        <v>10</v>
+        <v>STATUS</v>
       </c>
       <c r="E29" t="str">
-        <v>Applied Voltage (kV)</v>
+        <v>RESULT</v>
       </c>
       <c r="F29" t="str">
-        <v>80</v>
+        <v/>
       </c>
       <c r="G29" t="str">
-        <v>Exposure Time (s)</v>
+        <v/>
       </c>
       <c r="H29" t="str">
-        <v>1.0</v>
+        <v/>
       </c>
       <c r="I29" t="str">
-        <v>Workload (mA.min/week)</v>
+        <v/>
       </c>
       <c r="J29" t="str">
-        <v>100</v>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>LOCATION</v>
+        <v>Control Console</v>
       </c>
       <c r="B30" t="str">
-        <v>MAX. RADIATION LEVEL (MR/HR)</v>
+        <v>0.05</v>
       </c>
       <c r="C30" t="str">
-        <v>MR/WEEK</v>
+        <v/>
       </c>
       <c r="D30" t="str">
-        <v>STATUS</v>
+        <v/>
       </c>
       <c r="E30" t="str">
-        <v>RESULT</v>
+        <v>Worker</v>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Control Console</v>
+        <v>Waiting Area</v>
       </c>
       <c r="B31" t="str">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="C31" t="str">
         <v/>
@@ -1409,29 +2711,27 @@
         <v/>
       </c>
       <c r="E31" t="str">
-        <v>Worker</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>Waiting Area</v>
-      </c>
-      <c r="B32" t="str">
-        <v>0.02</v>
-      </c>
-      <c r="C32" t="str">
-        <v/>
-      </c>
-      <c r="D32" t="str">
-        <v/>
-      </c>
-      <c r="E32" t="str">
         <v>Public</v>
+      </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+      <c r="H31" t="str">
+        <v/>
+      </c>
+      <c r="I31" t="str">
+        <v/>
+      </c>
+      <c r="J31" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add new dental CBCT and OPG templates with updated test data formats
- Introduced new templates for Dental CBCT and OPG, including both timer and no-timer variations.
- Updated test data formats to enhance clarity and consistency across various tests, including accuracy of operating potential and total filtration.
- Improved organization of test parameters and results for better usability in reporting and data handling.
</commit_message>
<xml_diff>
--- a/public/templates/Dental_CBCT_Template.xlsx
+++ b/public/templates/Dental_CBCT_Template.xlsx
@@ -543,7 +543,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>FCD</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B14" t="str">
         <v>100</v>
@@ -552,24 +552,27 @@
         <v>kV</v>
       </c>
       <c r="D14" t="str">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E14" t="str">
         <v>mA</v>
       </c>
       <c r="F14" t="str">
-        <v>10</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Set Time (mSec)</v>
+        <v>Set Time (ms)</v>
       </c>
       <c r="B15" t="str">
-        <v>Measured Time (mSec)</v>
+        <v>Measured Time 1 (ms)</v>
       </c>
       <c r="C15" t="str">
-        <v>% Error</v>
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Tolerance Value (%)</v>
       </c>
     </row>
     <row r="16">
@@ -577,10 +580,13 @@
         <v>100</v>
       </c>
       <c r="B16" t="str">
-        <v>102</v>
+        <v>98.5</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>&lt;=</v>
+      </c>
+      <c r="D16" t="str">
+        <v>20</v>
       </c>
     </row>
     <row r="17">
@@ -590,9 +596,6 @@
       <c r="B17" t="str">
         <v>198</v>
       </c>
-      <c r="C17" t="str">
-        <v/>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -601,7 +604,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>FCD</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B20" t="str">
         <v>100</v>
@@ -610,10 +613,10 @@
         <v>kV</v>
       </c>
       <c r="D20" t="str">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E20" t="str">
-        <v>Timer</v>
+        <v>Time (s)</v>
       </c>
       <c r="F20" t="str">
         <v>0.1</v>
@@ -621,78 +624,48 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Tolerance Operator</v>
+        <v>mA Applied</v>
       </c>
       <c r="B21" t="str">
-        <v>&lt;=</v>
+        <v>Measured Output 1</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Measured Output 2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Tolerance Value (CoL)</v>
+        <v>50</v>
       </c>
       <c r="B22" t="str">
-        <v>0.1</v>
+        <v>0.5</v>
+      </c>
+      <c r="C22" t="str">
+        <v>0.51</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>mA Station</v>
+        <v>100</v>
       </c>
       <c r="B23" t="str">
-        <v>Measured mR 1</v>
-      </c>
-      <c r="C23" t="str">
-        <v>Measured mR 2</v>
-      </c>
-      <c r="D23" t="str">
-        <v>Measured mR 3</v>
-      </c>
-      <c r="E23" t="str">
-        <v>Average</v>
-      </c>
-      <c r="F23" t="str">
-        <v>mR/mAs</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>10</v>
+        <v>Tolerance Operator</v>
       </c>
       <c r="B24" t="str">
-        <v>2.4</v>
-      </c>
-      <c r="C24" t="str">
-        <v>2.45</v>
-      </c>
-      <c r="D24" t="str">
-        <v>2.42</v>
-      </c>
-      <c r="E24" t="str">
-        <v/>
-      </c>
-      <c r="F24" t="str">
-        <v/>
+        <v>&lt;=</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>20</v>
+        <v>Tolerance Value (CoL)</v>
       </c>
       <c r="B25" t="str">
-        <v>4.8</v>
-      </c>
-      <c r="C25" t="str">
-        <v>4.85</v>
-      </c>
-      <c r="D25" t="str">
-        <v>4.82</v>
-      </c>
-      <c r="E25" t="str">
-        <v/>
-      </c>
-      <c r="F25" t="str">
-        <v/>
+        <v>0.1</v>
       </c>
     </row>
     <row r="27">
@@ -702,78 +675,54 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Tolerance Operator</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B28" t="str">
-        <v>&lt;=</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Tolerance Value (CoV)</v>
+        <v>kVp</v>
       </c>
       <c r="B29" t="str">
-        <v>0.05</v>
+        <v>mAs</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Output 1</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Output 2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>FFD</v>
+        <v>80</v>
       </c>
       <c r="B30" t="str">
-        <v>100</v>
+        <v>10</v>
+      </c>
+      <c r="C30" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="D30" t="str">
+        <v>0.51</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>kVp</v>
+        <v>Tolerance Operator</v>
       </c>
       <c r="B31" t="str">
-        <v>mAs</v>
-      </c>
-      <c r="C31" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="D31" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="E31" t="str">
-        <v>Meas 3</v>
-      </c>
-      <c r="F31" t="str">
-        <v>Mean</v>
-      </c>
-      <c r="G31" t="str">
-        <v>CoV</v>
-      </c>
-      <c r="H31" t="str">
-        <v>Remarks</v>
+        <v>&lt;=</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>80</v>
+        <v>Tolerance Value (CoV)</v>
       </c>
       <c r="B32" t="str">
-        <v>100</v>
-      </c>
-      <c r="C32" t="str">
-        <v>10.2</v>
-      </c>
-      <c r="D32" t="str">
-        <v>10.1</v>
-      </c>
-      <c r="E32" t="str">
-        <v>10.3</v>
-      </c>
-      <c r="F32" t="str">
-        <v/>
-      </c>
-      <c r="G32" t="str">
-        <v/>
-      </c>
-      <c r="H32" t="str">
-        <v/>
+        <v>0.05</v>
       </c>
     </row>
     <row r="34">
@@ -824,24 +773,27 @@
         <v>Location</v>
       </c>
       <c r="B36" t="str">
-        <v>Front</v>
+        <v>Left</v>
       </c>
       <c r="C36" t="str">
-        <v>Back</v>
+        <v>Right</v>
       </c>
       <c r="D36" t="str">
-        <v>Left</v>
+        <v>Top</v>
       </c>
       <c r="E36" t="str">
-        <v>Right</v>
+        <v>Up</v>
       </c>
       <c r="F36" t="str">
+        <v>Down</v>
+      </c>
+      <c r="G36" t="str">
         <v>Max Leakage</v>
       </c>
-      <c r="G36" t="str">
+      <c r="H36" t="str">
         <v>Unit</v>
       </c>
-      <c r="H36" t="str">
+      <c r="I36" t="str">
         <v>Remark</v>
       </c>
     </row>
@@ -862,12 +814,15 @@
         <v>0.011</v>
       </c>
       <c r="F37" t="str">
-        <v/>
+        <v>0.010</v>
       </c>
       <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
         <v>mGy/h</v>
       </c>
-      <c r="H37" t="str">
+      <c r="I37" t="str">
         <v/>
       </c>
     </row>
@@ -888,12 +843,15 @@
         <v>0.013</v>
       </c>
       <c r="F38" t="str">
-        <v/>
+        <v>0.012</v>
       </c>
       <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
         <v>mGy/h</v>
       </c>
-      <c r="H38" t="str">
+      <c r="I38" t="str">
         <v/>
       </c>
     </row>
@@ -988,7 +946,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L39"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1133,104 +1091,98 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Tolerance Operator</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B14" t="str">
-        <v>&lt;=</v>
+        <v>100</v>
+      </c>
+      <c r="C14" t="str">
+        <v>kV</v>
+      </c>
+      <c r="D14" t="str">
+        <v>80</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Tolerance Value (CoL)</v>
+        <v>mAs Range</v>
       </c>
       <c r="B15" t="str">
-        <v>0.1</v>
+        <v>Measured Output 1</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Measured Output 2</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Measured Output 3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>mAs Range</v>
+        <v>5 - 10</v>
       </c>
       <c r="B16" t="str">
-        <v>Measured mR 1</v>
+        <v>0.5</v>
       </c>
       <c r="C16" t="str">
-        <v>Measured mR 2</v>
+        <v>0.51</v>
       </c>
       <c r="D16" t="str">
-        <v>Measured mR 3</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Average</v>
-      </c>
-      <c r="F16" t="str">
-        <v>mR/mAs</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>50</v>
+        <v>10 - 20</v>
       </c>
       <c r="B17" t="str">
-        <v>12.2</v>
+        <v>1</v>
       </c>
       <c r="C17" t="str">
-        <v>12.25</v>
+        <v>1.01</v>
       </c>
       <c r="D17" t="str">
-        <v>12.22</v>
-      </c>
-      <c r="E17" t="str">
-        <v/>
-      </c>
-      <c r="F17" t="str">
-        <v/>
+        <v>0.99</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>100</v>
+        <v>20 - 50</v>
       </c>
       <c r="B18" t="str">
-        <v>24.4</v>
+        <v>2.5</v>
       </c>
       <c r="C18" t="str">
-        <v>24.45</v>
+        <v>2.51</v>
       </c>
       <c r="D18" t="str">
-        <v>24.42</v>
-      </c>
-      <c r="E18" t="str">
-        <v/>
-      </c>
-      <c r="F18" t="str">
-        <v/>
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="B19" t="str">
+        <v>&lt;=</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>TEST: CONSISTENCY OF RADIATION OUTPUT</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Tolerance Operator</v>
-      </c>
-      <c r="B21" t="str">
-        <v>&lt;=</v>
+        <v>Tolerance Value (CoL)</v>
+      </c>
+      <c r="B20" t="str">
+        <v>0.1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Tolerance Value (CoV)</v>
-      </c>
-      <c r="B22" t="str">
-        <v>0.05</v>
+        <v>TEST: CONSISTENCY OF RADIATION OUTPUT</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>FFD</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B23" t="str">
         <v>100</v>
@@ -1244,22 +1196,10 @@
         <v>mAs</v>
       </c>
       <c r="C24" t="str">
-        <v>Meas 1</v>
+        <v>Output 1</v>
       </c>
       <c r="D24" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="E24" t="str">
-        <v>Meas 3</v>
-      </c>
-      <c r="F24" t="str">
-        <v>Mean</v>
-      </c>
-      <c r="G24" t="str">
-        <v>CoV</v>
-      </c>
-      <c r="H24" t="str">
-        <v>Remarks</v>
+        <v>Output 2</v>
       </c>
     </row>
     <row r="25">
@@ -1267,233 +1207,246 @@
         <v>80</v>
       </c>
       <c r="B25" t="str">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C25" t="str">
-        <v>10.2</v>
+        <v>0.5</v>
       </c>
       <c r="D25" t="str">
-        <v>10.1</v>
-      </c>
-      <c r="E25" t="str">
-        <v>10.3</v>
-      </c>
-      <c r="F25" t="str">
-        <v/>
-      </c>
-      <c r="G25" t="str">
-        <v/>
-      </c>
-      <c r="H25" t="str">
-        <v/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="B26" t="str">
+        <v>&lt;=</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>TEST: RADIATION LEAKAGE LEVEL FROM X-RAY TUBE HOUSE</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>kV</v>
-      </c>
-      <c r="B28" t="str">
-        <v>120</v>
-      </c>
-      <c r="C28" t="str">
-        <v>mA</v>
-      </c>
-      <c r="D28" t="str">
-        <v>10</v>
-      </c>
-      <c r="E28" t="str">
-        <v>Time</v>
-      </c>
-      <c r="F28" t="str">
-        <v>1.0</v>
-      </c>
-      <c r="G28" t="str">
-        <v>Workload</v>
-      </c>
-      <c r="H28" t="str">
-        <v>100</v>
-      </c>
-      <c r="I28" t="str">
-        <v>Tolerance</v>
-      </c>
-      <c r="J28" t="str">
-        <v>1.0</v>
-      </c>
-      <c r="K28" t="str">
-        <v>Tolerance Operator</v>
-      </c>
-      <c r="L28" t="str">
-        <v>&lt;</v>
+        <v>Tolerance Value (CoV)</v>
+      </c>
+      <c r="B27" t="str">
+        <v>0.05</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Location</v>
-      </c>
-      <c r="B29" t="str">
-        <v>Front</v>
-      </c>
-      <c r="C29" t="str">
-        <v>Back</v>
-      </c>
-      <c r="D29" t="str">
-        <v>Left</v>
-      </c>
-      <c r="E29" t="str">
-        <v>Right</v>
-      </c>
-      <c r="F29" t="str">
-        <v>Max Leakage</v>
-      </c>
-      <c r="G29" t="str">
-        <v>Unit</v>
-      </c>
-      <c r="H29" t="str">
-        <v>Remark</v>
+        <v>TEST: RADIATION LEAKAGE LEVEL FROM X-RAY TUBE HOUSE</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Tube</v>
+        <v>kV</v>
       </c>
       <c r="B30" t="str">
-        <v>0.01</v>
+        <v>120</v>
       </c>
       <c r="C30" t="str">
-        <v>0.015</v>
+        <v>mA</v>
       </c>
       <c r="D30" t="str">
-        <v>0.012</v>
+        <v>10</v>
       </c>
       <c r="E30" t="str">
-        <v>0.011</v>
+        <v>Time</v>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>1.0</v>
       </c>
       <c r="G30" t="str">
-        <v>mGy/h</v>
+        <v>Workload</v>
       </c>
       <c r="H30" t="str">
-        <v/>
+        <v>100</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Tolerance</v>
+      </c>
+      <c r="J30" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="L30" t="str">
+        <v>&lt;</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Collimator</v>
+        <v>Location</v>
       </c>
       <c r="B31" t="str">
+        <v>Left</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Right</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Top</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Up</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Down</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Max Leakage</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Remark</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Tube</v>
+      </c>
+      <c r="B32" t="str">
+        <v>0.01</v>
+      </c>
+      <c r="C32" t="str">
+        <v>0.015</v>
+      </c>
+      <c r="D32" t="str">
         <v>0.012</v>
       </c>
-      <c r="C31" t="str">
+      <c r="E32" t="str">
         <v>0.011</v>
       </c>
-      <c r="D31" t="str">
-        <v>0.014</v>
-      </c>
-      <c r="E31" t="str">
-        <v>0.013</v>
-      </c>
-      <c r="F31" t="str">
-        <v/>
-      </c>
-      <c r="G31" t="str">
+      <c r="F32" t="str">
+        <v>0.010</v>
+      </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
+      <c r="H32" t="str">
         <v>mGy/h</v>
       </c>
-      <c r="H31" t="str">
+      <c r="I32" t="str">
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>TEST: RADIATION PROTECTION SURVEY REPORT</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>Applied Current (mA)</v>
-      </c>
-      <c r="B34" t="str">
-        <v>10</v>
-      </c>
-      <c r="C34" t="str">
-        <v>Applied Voltage (kV)</v>
-      </c>
-      <c r="D34" t="str">
-        <v>80</v>
-      </c>
-      <c r="E34" t="str">
-        <v>Exposure Time (s)</v>
-      </c>
-      <c r="F34" t="str">
-        <v>1.0</v>
-      </c>
-      <c r="G34" t="str">
-        <v>Workload (mA.min/week)</v>
-      </c>
-      <c r="H34" t="str">
-        <v>100</v>
+        <v>Collimator</v>
+      </c>
+      <c r="B33" t="str">
+        <v>0.012</v>
+      </c>
+      <c r="C33" t="str">
+        <v>0.011</v>
+      </c>
+      <c r="D33" t="str">
+        <v>0.014</v>
+      </c>
+      <c r="E33" t="str">
+        <v>0.013</v>
+      </c>
+      <c r="F33" t="str">
+        <v>0.012</v>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
+        <v>mGy/h</v>
+      </c>
+      <c r="I33" t="str">
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>LOCATION</v>
-      </c>
-      <c r="B35" t="str">
-        <v>MAX. RADIATION LEVEL (MR/HR)</v>
-      </c>
-      <c r="C35" t="str">
-        <v>MR/WEEK</v>
-      </c>
-      <c r="D35" t="str">
-        <v>STATUS</v>
-      </c>
-      <c r="E35" t="str">
-        <v>RESULT</v>
+        <v>TEST: RADIATION PROTECTION SURVEY REPORT</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Control Console</v>
+        <v>Applied Current (mA)</v>
       </c>
       <c r="B36" t="str">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="C36" t="str">
-        <v/>
+        <v>Applied Voltage (kV)</v>
       </c>
       <c r="D36" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="E36" t="str">
-        <v>Worker</v>
+        <v>Exposure Time (s)</v>
+      </c>
+      <c r="F36" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Workload (mA.min/week)</v>
+      </c>
+      <c r="H36" t="str">
+        <v>100</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
+        <v>LOCATION</v>
+      </c>
+      <c r="B37" t="str">
+        <v>MAX. RADIATION LEVEL (MR/HR)</v>
+      </c>
+      <c r="C37" t="str">
+        <v>MR/WEEK</v>
+      </c>
+      <c r="D37" t="str">
+        <v>STATUS</v>
+      </c>
+      <c r="E37" t="str">
+        <v>RESULT</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Control Console</v>
+      </c>
+      <c r="B38" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="C38" t="str">
+        <v/>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v>Worker</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
         <v>Waiting Area</v>
       </c>
-      <c r="B37" t="str">
+      <c r="B39" t="str">
         <v>0.02</v>
       </c>
-      <c r="C37" t="str">
-        <v/>
-      </c>
-      <c r="D37" t="str">
-        <v/>
-      </c>
-      <c r="E37" t="str">
+      <c r="C39" t="str">
+        <v/>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
         <v>Public</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L39"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>